<commit_message>
Take West Kazakhstan out of the model perimeter
The West (Atyrau, Mangystau) is a gas island synchronous with Russia and
cannot trade with CAPS. The 2020 model folded its load into KAZ_N without
its plants, which overstated the tightness of the North by 16 TWh.

zones_demand.csv gains a scope column: an excluded zone keeps its share of
the national energy, so the zones that stay are not inflated by it, but it
is not written out. KAZ_N 64.4 %, KAZ_S 22.7 %, out of perimeter 12.9 %.

Also on the documentation page: the country matrix comes first, and the
five French source ids are renamed (equipe, hypothese, gabarit_2026,
demande_tso, courriels_equipe).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_build/DATA_SOURCES_casa.xlsx
+++ b/data_build/DATA_SOURCES_casa.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>equipe</t>
+          <t>team</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr"/>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>deca_v51, gabarit_2026</t>
+          <t>deca_v51, template_2026</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>Filled by extract_demand.py, DeCA Reference scenario. Demand Evolution covers 2023-2060 BY COUNTRY: no extrapolation is needed for Central Asia. The intra- country split comes from the 8760 h profiles and stays constant over time, DeCA giving no regional trajectory. The zonal peak is NON COINCIDENT, as required by generate_demand.gms which multiplies it by the normalised profile of the zone: the own peak is therefore rescaled by the growth of the country peak, through the observed coincidence factor (KG 1.03, KZ 1.02, TJ 1.07, TM and UZ 1.00). Three deliberate departures, all documented in mappings/zones_demand.csv: the Tajik split is REVERSED with respect to the 2020 model (North 27.7 % against 74.9 %), the Kyrgyz split too (North 63.9 % against 93.2 %), and Western Kazakhstan is attached to KAZ_N for want of a third zone. The peak block of the TJ book was in GW under a MW label: corrected by a generic guard, a peak not being allowed to fall below the average power. AFG and PAK have no 2026 source: carried over from the 2020 pDemandData and extended at their own rate, LOW confidence.</t>
+          <t>Filled by extract_demand.py, DeCA Reference scenario. Demand Evolution covers 2023-2060 BY COUNTRY: no extrapolation is needed for Central Asia. The intra- country split comes from the 8760 h profiles and stays constant over time, DeCA giving no regional trajectory. The zonal peak is NON COINCIDENT, as required by generate_demand.gms which multiplies it by the normalised profile of the zone: the own peak is therefore rescaled by the growth of the country peak, through the observed coincidence factor (KG 1.03, KZ 1.02, TJ 1.07, TM and UZ 1.00). Three deliberate departures, all documented in mappings/zones_demand.csv: the Tajik split is REVERSED with respect to the 2020 model (North 27.7 % against 74.9 %), the Kyrgyz split too (North 63.9 % against 93.2 %), and Western Kazakhstan is OUT OF PERIMETER. The West (Atyrau, Mangystau) is a gas island synchronous with Russia, unable to trade with CAPS; the 2020 model folded its load into KAZ_N without its plants, which overstated the tightness of the North. It keeps its 12.9 % share of the national energy so that the North and the South are not inflated by it, and is dropped from the output: the KZ split is KAZ_N 64.4 %, KAZ_S 22.7 %, out of perimeter 12.9 %. Modelled Kazakhstan is North plus South, about 87 % of national consumption, which is what the results must be read against. The peak block of the TJ book was in GW under a MW label: corrected by a generic guard, a peak not being allowed to fall below the average power. AFG and PAK have no 2026 source: carried over from the 2020 pDemandData and extended at their own rate, LOW confidence.</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>deca_v51, gabarit_2026</t>
+          <t>deca_v51, template_2026</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>hypothese</t>
+          <t>assumed</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr"/>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>deca_v51, hypothese</t>
+          <t>deca_v51, assumed</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>deca_v51, demande_tso</t>
+          <t>deca_v51, tso_request</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>hypothese</t>
+          <t>assumed</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr"/>
@@ -3163,7 +3163,7 @@
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>hypothese</t>
+          <t>assumed</t>
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr"/>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>hypothese</t>
+          <t>assumed</t>
         </is>
       </c>
       <c r="K52" s="4" t="inlineStr"/>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>hypothese</t>
+          <t>assumed</t>
         </is>
       </c>
       <c r="K53" s="4" t="inlineStr"/>
@@ -3697,7 +3697,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>gabarit_2026</t>
+          <t>template_2026</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -3981,7 +3981,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>demande_tso</t>
+          <t>tso_request</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -4047,7 +4047,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>equipe</t>
+          <t>team</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -4076,7 +4076,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>hypothese</t>
+          <t>assumed</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -4109,7 +4109,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>courriels_equipe</t>
+          <t>team_emails</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Record the Renewables.ninja fetch in the source registry
Marks the entry TESTED - FETCHED with what was actually fetched -- 2022, sixteen
zones, both technologies, relabelled to zone local time -- and with the two numbers
a reader needs before trusting it: solar reads about 22 per cent above the profiles
now in the model, and the wind levels disagree with the model about which zones are
windy rather than by a constant. The verdict is written down rather than left to be
rediscovered: take the shape, keep DeCA's level, and get Global Wind Atlas for the
wind resource.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_build/DATA_SOURCES_casa.xlsx
+++ b/data_build/DATA_SOURCES_casa.xlsx
@@ -4127,7 +4127,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Hourly solar and wind profiles by coordinates. Already used by pre-analysis/pipelines/vre_pipeline.py.</t>
+          <t>Hourly solar and wind profiles by coordinates. FETCHED: 2022, one year, all sixteen zones and both technologies, by pre-analysis/pipelines/run_casa_vre_fetch.py. Two things to know before using it. THE LEVEL IS NOT DECA'S. Solar comes out 3 to 46 per cent above the profiles now in the model, mean 0.204 against 0.167, which is what a clean modelled array with a flat ten per cent loss does against metered output carrying outages, soiling and curtailment. Wind does not differ by a level at all but by which zones are windy: the model gives every zone 0.33 to 0.42, a placeholder, while this says Herat 0.63, Kazakhstan 0.51 and the mountain zones near zero, TAJ_S at 0.016. The ranking is physically right and the model's flat value is wrong, but neither number is usable as a level -- the default turbine is a low specific power machine that reads high by design, and MERRA-2 at half a degree cannot resolve a Pamir valley at all. USE THE SHAPE, KEEP DECA'S LEVEL. THE COORDINATES ARE POLYGON POINTS, one per zone, from data_build/build_vre_coords.py, because no plant in the fleet carries a latitude anywhere. Global Wind Atlas at one kilometre is the source that would settle the wind level properly.</t>
         </is>
       </c>
     </row>
@@ -4939,19 +4939,19 @@
           <t>renewables.ninja, globalwindatlas.info</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>TESTED - AVAILABLE</t>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>TESTED - FETCHED</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Hourly solar and wind profiles simulated anywhere on the globe from the ERA5 reanalysis.</t>
+          <t>Hourly solar and wind profiles simulated anywhere on the globe. FETCHED for 2022, sixteen zones, both technologies, 8760 h each, relabelled to zone local time. Held outside the repo in pre-analysis/representative_days/input as PV_casa.csv and WT_casa.csv.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>The only route to pVREProfile in Turkmenistan, in Afghanistan and wherever DeCA gives nothing. Already wired into pre-analysis/pipelines/vre_pipeline.py.</t>
+          <t>The route out of the pVREProfile staircase, and the only route at all in Turkmenistan and Afghanistan. Take the SHAPE and keep the DeCA level: solar reads 22 per cent high on average and the wind levels are a turbine-model artifact over a half-degree grid. Global Wind Atlas, still untested, is what would settle the wind level.</t>
         </is>
       </c>
     </row>

</xml_diff>